<commit_message>
Subcomponentes sobre consolidada total con evidencia y llaves; dedup columnas
- subcomponentes_consolidado.py: aplica los 17 subcomponentes de cierre de
  brecha a TODOS los cod_local de la base consolidada (11 grupos), validando con
  Rep_Activos_F7 (activo por CUI) + HR Inversiones (componentes por CUI).
- subcomponentes_total_matriz (59,144 x 28): 1/0 por subcomponente por cod_local,
  con llaves (cui, cod_modular), grupos, total cumplidos, activos_f7 y estado.
- subcomponentes_total_evidencia (1,005,448 filas): por (cod_local,
  subcomponente) adjunta activo_que_valida y la variable ESTADO para cotejo.
- Pipeline principal: elimina columnas con contenido duplicado en cada base
  individual (cada variable aparece una sola vez). Regenera todas las salidas.

https://claude.ai/code/session_01N9afypBcQVKYhttom8P34Z
</commit_message>
<xml_diff>
--- a/output/bases_limpias/Grupo_03_MODULOS/df_ugrd_mbr.xlsx
+++ b/output/bases_limpias/Grupo_03_MODULOS/df_ugrd_mbr.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z61"/>
+  <dimension ref="A1:Y61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,60 +489,55 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>fecha_de_inauguracion_o_estimada</t>
+          <t>comentario</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>comentario</t>
+          <t>departamento</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>departamento</t>
+          <t>provincia</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>provincia</t>
+          <t>distrito</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>distrito</t>
+          <t>centro_poblado</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>centro_poblado</t>
+          <t>ubigeo</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>ubigeo</t>
+          <t>dre</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>dre</t>
+          <t>ugel</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>ugel</t>
+          <t>nombre_ie</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>nombre_ie</t>
+          <t>area</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
-        <is>
-          <t>area</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
         <is>
           <t>fuente</t>
         </is>
@@ -605,58 +600,57 @@
           <t>27/08/2024</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>MORROPON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>MORROPON</t>
+          <t>YAMANGO</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>YAMANGO</t>
+          <t>SAN CRISTOBAL</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>SAN CRISTOBAL</t>
+          <t>200410</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>200410</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL MORROPÓN</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>UGEL MORROPÓN</t>
+          <t>14687</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>14687</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -719,20 +713,24 @@
           <t>29/09/2023</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LA LIBERTAD</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>LA LIBERTAD</t>
+          <t>TRUJILLO</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>TRUJILLO</t>
+          <t>HUANCHACO</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -742,35 +740,30 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>HUANCHACO</t>
+          <t>130104</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>130104</t>
+          <t>GRE LA LIBERTAD</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>GRE LA LIBERTAD</t>
+          <t>UGEL 02 - LA ESPERANZA</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>UGEL 02 - LA ESPERANZA</t>
+          <t>2270</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2270</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -833,58 +826,57 @@
           <t>26/05/2023</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>SULLANA</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>SULLANA</t>
+          <t>LANCONES</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>LANCONES</t>
+          <t>CASAS QUEMADAS</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>CASAS QUEMADAS</t>
+          <t>200604</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>200604</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL SULLANA</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>UGEL SULLANA</t>
+          <t>14803/14803</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>14803/14803</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -947,20 +939,24 @@
           <t>27/04/2023</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LA LIBERTAD</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>LA LIBERTAD</t>
+          <t>TRUJILLO</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>TRUJILLO</t>
+          <t>LA ESPERANZA</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -970,35 +966,30 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>LA ESPERANZA</t>
+          <t>130105</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>130105</t>
+          <t>GRE LA LIBERTAD</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>GRE LA LIBERTAD</t>
+          <t>UGEL 02 - LA ESPERANZA</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>UGEL 02 - LA ESPERANZA</t>
+          <t>2311</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2311</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1061,20 +1052,24 @@
           <t>09/05/2023</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LAMBAYEQUE</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>LAMBAYEQUE</t>
+          <t>CHICLAYO</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>CHICLAYO</t>
+          <t>JOSE LEONARDO ORTIZ</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1084,35 +1079,30 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>JOSE LEONARDO ORTIZ</t>
+          <t>140105</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>140105</t>
+          <t>GRE LAMBAYEQUE</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>GRE LAMBAYEQUE</t>
+          <t>UGEL CHICLAYO</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>UGEL CHICLAYO</t>
+          <t>410</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1175,20 +1165,24 @@
           <t>18/04/2023</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LAMBAYEQUE</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>LAMBAYEQUE</t>
+          <t>CHICLAYO</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>CHICLAYO</t>
+          <t>JOSE LEONARDO ORTIZ</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1198,35 +1192,30 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>JOSE LEONARDO ORTIZ</t>
+          <t>140105</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>140105</t>
+          <t>GRE LAMBAYEQUE</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>GRE LAMBAYEQUE</t>
+          <t>UGEL CHICLAYO</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>UGEL CHICLAYO</t>
+          <t>436 LOS ANGELITOS DE SAN JUAN DE DIOS</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>436 LOS ANGELITOS DE SAN JUAN DE DIOS</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1289,20 +1278,24 @@
           <t>17/02/2023</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LA LIBERTAD</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>LA LIBERTAD</t>
+          <t>TRUJILLO</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>TRUJILLO</t>
+          <t>HUANCHACO</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1312,35 +1305,30 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>HUANCHACO</t>
+          <t>130104</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>130104</t>
+          <t>GRE LA LIBERTAD</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>GRE LA LIBERTAD</t>
+          <t>UGEL 02 - LA ESPERANZA</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>UGEL 02 - LA ESPERANZA</t>
+          <t>2209</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2209</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1403,58 +1391,57 @@
           <t>08/08/2023</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LAMBAYEQUE</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>LAMBAYEQUE</t>
+          <t>CHICLAYO</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>CHICLAYO</t>
+          <t>PATAPO</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>PATAPO</t>
+          <t>LAS CANTERAS</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>LAS CANTERAS</t>
+          <t>140117</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>140117</t>
+          <t>GRE LAMBAYEQUE</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>GRE LAMBAYEQUE</t>
+          <t>UGEL CHICLAYO</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>UGEL CHICLAYO</t>
+          <t>MARIA CESPEDES SIGNOL</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>MARIA CESPEDES SIGNOL</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z9" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1517,10 +1504,14 @@
           <t>26/10/2023</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1535,40 +1526,35 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>EL MOLINO</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>EL MOLINO</t>
+          <t>200101</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>200101</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL PIURA</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>UGEL PIURA</t>
+          <t>20137/20137</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>20137/20137</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1631,15 +1617,19 @@
           <t>05/12/2024</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>AIJA</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1654,35 +1644,30 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>AIJA</t>
+          <t>020201</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>020201</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL AIJA</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>UGEL AIJA</t>
+          <t>86135</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>86135</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1745,58 +1730,57 @@
           <t>12/09/2023</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>YUNGAY</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>YUNGAY</t>
+          <t>QUILLO</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>QUILLO</t>
+          <t>LA PALMA</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>LA PALMA</t>
+          <t>022005</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>022005</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL YUNGAY</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>UGEL YUNGAY</t>
+          <t>86653</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>86653</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1859,10 +1843,14 @@
           <t>08/03/2024</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1872,45 +1860,40 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>TAMBO GRANDE</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>TAMBO GRANDE</t>
+          <t>CP-16 JESUS MARIA</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>CP-16 JESUS MARIA</t>
+          <t>200114</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>200114</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL TAMBOGRANDE</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>UGEL TAMBOGRANDE</t>
+          <t>1437</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>1437</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -1973,20 +1956,24 @@
           <t>19/06/2025</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>AIJA</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>AIJA</t>
+          <t>HUACLLAN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1996,35 +1983,30 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>HUACLLAN</t>
+          <t>020203</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>020203</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL AIJA</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>UGEL AIJA</t>
+          <t>86161/86161</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>86161/86161</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z14" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2087,15 +2069,19 @@
           <t>22/11/2024</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LAMBAYEQUE</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>LAMBAYEQUE</t>
+          <t>CHICLAYO</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2110,35 +2096,30 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>CHICLAYO</t>
+          <t>140101</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>140101</t>
+          <t>GRE LAMBAYEQUE</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>GRE LAMBAYEQUE</t>
+          <t>UGEL CHICLAYO</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>UGEL CHICLAYO</t>
+          <t>10024 NUESTRA SEÑORA DE FATIMA/10024 NUESTRA SEÑORA DE FATIMA/10024 NUESTRA SEÑORA DE FATIMA</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>10024 NUESTRA SEÑORA DE FATIMA/10024 NUESTRA SEÑORA DE FATIMA/10024 NUESTRA SEÑORA DE FATIMA</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2201,20 +2182,24 @@
           <t>27/02/2023</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LA LIBERTAD</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>LA LIBERTAD</t>
+          <t>TRUJILLO</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>TRUJILLO</t>
+          <t>HUANCHACO</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2224,35 +2209,30 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>HUANCHACO</t>
+          <t>130104</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>130104</t>
+          <t>GRE LA LIBERTAD</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>GRE LA LIBERTAD</t>
+          <t>UGEL 02 - LA ESPERANZA</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>UGEL 02 - LA ESPERANZA</t>
+          <t>2271</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2271</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2315,58 +2295,57 @@
           <t>22/02/2022</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>SANTA</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>SANTA</t>
+          <t>CHIMBOTE</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>CHIMBOTE</t>
+          <t>RINCONADA</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>RINCONADA</t>
+          <t>021801</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>021801</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL SANTA</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>UGEL SANTA</t>
+          <t>1610</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>1610</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z17" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2429,58 +2408,57 @@
           <t>08/08/2024</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>SANTA</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>SANTA</t>
+          <t>CHIMBOTE</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>CHIMBOTE</t>
+          <t>MIRAMAR BAJO</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>MIRAMAR BAJO</t>
+          <t>021801</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>021801</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL SANTA</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>UGEL SANTA</t>
+          <t>88005 CORAZON DE JESUS</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>88005 CORAZON DE JESUS</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z18" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2543,58 +2521,57 @@
           <t>28/11/2022</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>AIJA</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>AIJA</t>
+          <t>LA MERCED</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>LA MERCED</t>
+          <t>MALLAKAYAN / MALLUCALLAN</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>MALLAKAYAN / MALLUCALLAN</t>
+          <t>020204</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>020204</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL AIJA</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>UGEL AIJA</t>
+          <t>86145</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>86145</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z19" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2657,58 +2634,57 @@
           <t>22/04/2022</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>AIJA</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>AIJA</t>
+          <t>CORIS</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>CORIS</t>
+          <t>ALMIZCLE</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>ALMIZCLE</t>
+          <t>020202</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>020202</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL AIJA</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>UGEL AIJA</t>
+          <t>86710/86710</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>86710/86710</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2771,20 +2747,24 @@
           <t>10/03/2023</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LA LIBERTAD</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>LA LIBERTAD</t>
+          <t>TRUJILLO</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>TRUJILLO</t>
+          <t>HUANCHACO</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2794,35 +2774,30 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>HUANCHACO</t>
+          <t>130104</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>130104</t>
+          <t>GRE LA LIBERTAD</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>GRE LA LIBERTAD</t>
+          <t>UGEL 02 - LA ESPERANZA</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>UGEL 02 - LA ESPERANZA</t>
+          <t>2154</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2154</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z21" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2885,15 +2860,19 @@
           <t>23/06/2023</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LA LIBERTAD</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>LA LIBERTAD</t>
+          <t>VIRU</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2903,40 +2882,35 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>VIRU</t>
+          <t>HUANCAQUITO BAJO</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>HUANCAQUITO BAJO</t>
+          <t>131201</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>131201</t>
+          <t>GRE LA LIBERTAD</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>GRE LA LIBERTAD</t>
+          <t>UGEL VIRÚ</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>UGEL VIRÚ</t>
+          <t>1735</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>1735</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z22" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -2999,58 +2973,57 @@
           <t>03/07/2025</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>AYABACA</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>AYABACA</t>
+          <t>SICCHEZ</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>SICCHEZ</t>
+          <t>OXAHUAY</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>OXAHUAY</t>
+          <t>200209</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>200209</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL AYABACA</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>UGEL AYABACA</t>
+          <t>109</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z23" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -3113,10 +3086,14 @@
           <t>08/08/2025</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -3126,7 +3103,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>CATACAOS</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3136,35 +3113,30 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>CATACAOS</t>
+          <t>200105</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>200105</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL PIURA</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>UGEL PIURA</t>
+          <t>15324/15324/15324</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>15324/15324/15324</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z24" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -3227,10 +3199,14 @@
           <t>29/12/2023</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -3240,45 +3216,40 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>TAMBO GRANDE</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>TAMBO GRANDE</t>
+          <t>JESUS DEL VALLE</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>JESUS DEL VALLE</t>
+          <t>200114</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>200114</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL TAMBOGRANDE</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>UGEL TAMBOGRANDE</t>
+          <t>912</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>912</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z25" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -3341,10 +3312,14 @@
           <t>29/12/2023</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -3354,45 +3329,40 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>LA UNION</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>LA UNION</t>
+          <t>SANTA CRUZ</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>SANTA CRUZ</t>
+          <t>200110</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>200110</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL LA UNIÓN</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>UGEL LA UNIÓN</t>
+          <t>15367</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>15367</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z26" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -3455,20 +3425,24 @@
           <t>21/07/2023</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LAMBAYEQUE</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>LAMBAYEQUE</t>
+          <t>CHICLAYO</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>CHICLAYO</t>
+          <t>LA VICTORIA</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3478,35 +3452,30 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>LA VICTORIA</t>
+          <t>140106</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>140106</t>
+          <t>GRE LAMBAYEQUE</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>GRE LAMBAYEQUE</t>
+          <t>UGEL CHICLAYO</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>UGEL CHICLAYO</t>
+          <t>035 MARAVILLA DE JESUS</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>035 MARAVILLA DE JESUS</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z27" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -3569,10 +3538,14 @@
           <t>04/05/2023</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -3587,40 +3560,35 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>SANTA SARA</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>SANTA SARA</t>
+          <t>200101</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>200101</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL PIURA</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>UGEL PIURA</t>
+          <t>20148</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>20148</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z28" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -3683,10 +3651,14 @@
           <t>28/12/2023</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -3696,45 +3668,40 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>CASTILLA</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>CASTILLA</t>
+          <t>SAN MARTIN KM.30</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>SAN MARTIN KM.30</t>
+          <t>200104</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>200104</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL PIURA</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>UGEL PIURA</t>
+          <t>785</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>785</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z29" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -3797,58 +3764,57 @@
           <t>04/02/2025</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LIMA PROVINCIAS</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>LIMA PROVINCIAS</t>
+          <t>YAUYOS</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>YAUYOS</t>
+          <t>COLONIA</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>COLONIA</t>
+          <t>QUISQUE</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>QUISQUE</t>
+          <t>151011</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>151011</t>
+          <t>DRE LIMA PROVINCIAS</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>DRE LIMA PROVINCIAS</t>
+          <t>UGEL 13 YAUYOS</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>UGEL 13 YAUYOS</t>
+          <t>20723/20723</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>20723/20723</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z30" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -3911,58 +3877,57 @@
           <t>23/05/2025</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>TALARA</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
+          <t>PARIÑAS</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
           <t>TALARA</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>PARIÑAS</t>
-        </is>
-      </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>TALARA</t>
+          <t>200701</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>200701</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL TALARA</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>UGEL TALARA</t>
+          <t>15038 SANTA ROSA DE LIMA/15038 SANTA ROSA DE LIMA/15038 SANTA ROSA DE LIMA</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>15038 SANTA ROSA DE LIMA/15038 SANTA ROSA DE LIMA/15038 SANTA ROSA DE LIMA</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z31" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4025,58 +3990,57 @@
           <t>13/05/2022</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>CASMA</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>CASMA</t>
+          <t>BUENA VISTA ALTA</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>BUENA VISTA ALTA</t>
+          <t>HACIENDA HUANCHUY</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>HACIENDA HUANCHUY</t>
+          <t>020802</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>020802</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL CASMA</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>UGEL CASMA</t>
+          <t>1583</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>1583</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z32" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4139,20 +4103,24 @@
           <t>28/03/2025</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>AIJA</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>AIJA</t>
+          <t>CORIS</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4162,35 +4130,30 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>CORIS</t>
+          <t>020202</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>020202</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL AIJA</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>UGEL AIJA</t>
+          <t>86153</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>86153</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z33" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4253,58 +4216,57 @@
           <t>26/08/2022</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>SECHURA</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>SECHURA</t>
+          <t>RINCONADA LLICUAR</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>RINCONADA LLICUAR</t>
+          <t>LLICUAR</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>LLICUAR</t>
+          <t>200806</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>200806</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL SECHURA</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>UGEL SECHURA</t>
+          <t>14073</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>14073</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z34" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4367,10 +4329,14 @@
           <t>05/03/2024</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4380,7 +4346,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>LA UNION</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4390,35 +4356,30 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>LA UNION</t>
+          <t>200110</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>200110</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL LA UNIÓN</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>UGEL LA UNIÓN</t>
+          <t>755</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>755</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z35" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4481,15 +4442,19 @@
           <t>04/12/2024</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>CORONGO</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -4504,35 +4469,30 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>CORONGO</t>
+          <t>020901</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>020901</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL CORONGO</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>UGEL CORONGO</t>
+          <t>88127</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>88127</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z36" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4595,15 +4555,19 @@
           <t>18/02/2022</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>SECHURA</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -4613,40 +4577,35 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>SECHURA</t>
+          <t>LA BOCANA/PARACHIQUE</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>LA BOCANA/PARACHIQUE</t>
+          <t>200801</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>200801</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL SECHURA</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>UGEL SECHURA</t>
+          <t>14083 MARIA VICTORIA RUMICHE FIESTAS DE MARTINEZ/14083 MARIA VICTORIA RUMICHE FIESTAS DE MARTINEZ</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>14083 MARIA VICTORIA RUMICHE FIESTAS DE MARTINEZ/14083 MARIA VICTORIA RUMICHE FIESTAS DE MARTINEZ</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z37" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4709,58 +4668,57 @@
           <t>24/05/2023</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>SECHURA</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>SECHURA</t>
+          <t>CRISTO NOS VALGA</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>CRISTO NOS VALGA</t>
+          <t>CERRITOS</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>CERRITOS</t>
+          <t>200804</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>200804</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL SECHURA</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>UGEL SECHURA</t>
+          <t>14046</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>14046</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z38" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4823,10 +4781,14 @@
           <t>05/04/2023</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -4836,45 +4798,40 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>CATACAOS</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>CATACAOS</t>
+          <t>SAN PABLO</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>SAN PABLO</t>
+          <t>200105</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>200105</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL PIURA</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>UGEL PIURA</t>
+          <t>14893</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>14893</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z39" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -4937,20 +4894,24 @@
           <t>04/07/2024</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>YUNGAY</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>YUNGAY</t>
+          <t>YANAMA</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4960,35 +4921,30 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>YANAMA</t>
+          <t>022008</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>022008</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL YUNGAY</t>
         </is>
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>UGEL YUNGAY</t>
+          <t>1550</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>1550</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z40" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5051,10 +5007,14 @@
           <t>19/04/2024</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LAMBAYEQUE</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -5064,45 +5024,40 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>LAMBAYEQUE</t>
+          <t>OLMOS</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>OLMOS</t>
+          <t>IMPERIAL / R. DE BURRO</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>IMPERIAL / R. DE BURRO</t>
+          <t>140308</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>140308</t>
+          <t>GRE LAMBAYEQUE</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>GRE LAMBAYEQUE</t>
+          <t>UGEL LAMBAYEQUE</t>
         </is>
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>UGEL LAMBAYEQUE</t>
+          <t>10190</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>10190</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z41" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5165,10 +5120,14 @@
           <t>28/02/2024</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -5178,7 +5137,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>CATACAOS</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -5188,35 +5147,30 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>CATACAOS</t>
+          <t>200105</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>200105</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL PIURA</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>UGEL PIURA</t>
+          <t>20151</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>20151</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z42" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5279,10 +5233,14 @@
           <t>11/07/2025</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LAMBAYEQUE</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -5292,45 +5250,40 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>LAMBAYEQUE</t>
+          <t>MOTUPE</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>MOTUPE</t>
+          <t>SALITRAL</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>SALITRAL</t>
+          <t>140307</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>140307</t>
+          <t>GRE LAMBAYEQUE</t>
         </is>
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>GRE LAMBAYEQUE</t>
+          <t>UGEL LAMBAYEQUE</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>UGEL LAMBAYEQUE</t>
+          <t>10150 SANTOS CARDENAS VALLADARES/10150 SANTOS CARDENAS VALLADARES</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>10150 SANTOS CARDENAS VALLADARES/10150 SANTOS CARDENAS VALLADARES</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z43" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5393,58 +5346,57 @@
           <t>10/05/2024</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>SULLANA</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>SULLANA</t>
+          <t>LANCONES</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>LANCONES</t>
+          <t>HUASIMAL DE LOS ENCUENTROS</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>HUASIMAL DE LOS ENCUENTROS</t>
+          <t>200604</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>200604</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL SULLANA</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>UGEL SULLANA</t>
+          <t>15286</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>15286</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z44" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5507,15 +5459,19 @@
           <t>23/10/2025</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>YUNGAY</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -5525,40 +5481,35 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>YUNGAY</t>
+          <t>CAYASBAMBA</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>CAYASBAMBA</t>
+          <t>022001</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>022001</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL YUNGAY</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>UGEL YUNGAY</t>
+          <t>89539 SANTA ROSA DE CAYASBAMBA/89539 SANTA ROSA DE CAYASBAMBA</t>
         </is>
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>89539 SANTA ROSA DE CAYASBAMBA/89539 SANTA ROSA DE CAYASBAMBA</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y45" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z45" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5621,58 +5572,57 @@
           <t>12/12/2025</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>MORROPON</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>MORROPON</t>
+          <t>SALITRAL</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>SALITRAL</t>
+          <t>SAN PEDRO</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>SAN PEDRO</t>
+          <t>200406</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>200406</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL MORROPÓN</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>UGEL MORROPÓN</t>
+          <t>20225</t>
         </is>
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>20225</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y46" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z46" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5735,15 +5685,19 @@
           <t>21/08/2024</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>YUNGAY</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -5753,40 +5707,35 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>YUNGAY</t>
+          <t>ONGO</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>ONGO</t>
+          <t>022001</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>022001</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL YUNGAY</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>UGEL YUNGAY</t>
+          <t>86651</t>
         </is>
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>86651</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y47" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z47" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5849,58 +5798,57 @@
           <t>19/11/2025</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>HUARI</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>HUARI</t>
+          <t>HUACACHI</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>HUACACHI</t>
+          <t>LA MERCED</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>LA MERCED</t>
+          <t>021005</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>021005</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL HUARI</t>
         </is>
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>UGEL HUARI</t>
+          <t>86416</t>
         </is>
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>86416</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y48" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z48" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -5963,15 +5911,19 @@
           <t>28/11/2025</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>YUNGAY</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -5981,40 +5933,35 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>YUNGAY</t>
+          <t>CANCHARRUMI</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>CANCHARRUMI</t>
+          <t>022001</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>022001</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL YUNGAY</t>
         </is>
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>UGEL YUNGAY</t>
+          <t>86749/86749</t>
         </is>
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>86749/86749</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y49" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z49" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6077,58 +6024,57 @@
           <t>25/07/2023</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>SANTA</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>SANTA</t>
+          <t>NEPEÑA</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>NEPEÑA</t>
+          <t>SAN JUAN</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>SAN JUAN</t>
+          <t>021806</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>021806</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL SANTA</t>
         </is>
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>UGEL SANTA</t>
+          <t>88271/88271</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>88271/88271</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z50" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6191,20 +6137,24 @@
           <t>13/03/2025</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>AIJA</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>AIJA</t>
+          <t>CORIS</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -6214,35 +6164,30 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>CORIS</t>
+          <t>020202</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>020202</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL AIJA</t>
         </is>
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>UGEL AIJA</t>
+          <t>86153</t>
         </is>
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>86153</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y51" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z51" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6305,58 +6250,57 @@
           <t>21/11/2025</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>HUARAZ</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>HUARAZ</t>
+          <t>HUANCHAY</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>HUANCHAY</t>
+          <t>MAHUACANCHA</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>MAHUACANCHA</t>
+          <t>020104</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>020104</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL HUARMEY</t>
         </is>
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>UGEL HUARMEY</t>
+          <t>86057</t>
         </is>
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>86057</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y52" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z52" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6419,10 +6363,14 @@
           <t>13/12/2024</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -6432,7 +6380,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>LA UNION</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6442,35 +6390,30 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>LA UNION</t>
+          <t>200110</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>200110</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL LA UNIÓN</t>
         </is>
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>UGEL LA UNIÓN</t>
+          <t>14989</t>
         </is>
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>14989</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y53" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z53" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6533,58 +6476,57 @@
           <t>26/03/2024</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>SULLANA</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>SULLANA</t>
+          <t>LANCONES</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>LANCONES</t>
+          <t>LEONES</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>LEONES</t>
+          <t>200604</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>200604</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL SULLANA</t>
         </is>
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>UGEL SULLANA</t>
+          <t>15250/15250/15250</t>
         </is>
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>15250/15250/15250</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y54" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z54" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6647,10 +6589,14 @@
           <t>30/04/2026</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -6660,45 +6606,40 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
+          <t>VEINTISEIS DE OCTUBRE</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
           <t>PIURA</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t>VEINTISEIS DE OCTUBRE</t>
-        </is>
-      </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>200115</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>200115</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL PIURA</t>
         </is>
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>UGEL PIURA</t>
+          <t>016 EMILIA BARCIA BONIFFATTI</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>016 EMILIA BARCIA BONIFFATTI</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y55" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z55" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6761,58 +6702,57 @@
           <t>30/04/2026</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>AYABACA</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>AYABACA</t>
+          <t>FRIAS</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>FRIAS</t>
+          <t>SAN DIEGO</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>SAN DIEGO</t>
+          <t>200202</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>200202</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL CHULUCANAS</t>
         </is>
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>UGEL CHULUCANAS</t>
+          <t>20007</t>
         </is>
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>20007</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y56" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z56" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6875,58 +6815,57 @@
           <t>27/07/2026</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr"/>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>LIMA PROVINCIAS</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>LIMA PROVINCIAS</t>
+          <t>CAÑETE</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>CAÑETE</t>
+          <t>QUILMANA</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>QUILMANA</t>
+          <t>EL TIGRE</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>EL TIGRE</t>
+          <t>150512</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
         <is>
-          <t>150512</t>
+          <t>DRE LIMA PROVINCIAS</t>
         </is>
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>DRE LIMA PROVINCIAS</t>
+          <t>UGEL 08 CAÑETE</t>
         </is>
       </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>UGEL 08 CAÑETE</t>
+          <t>20176/20176</t>
         </is>
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>20176/20176</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y57" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z57" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -6989,58 +6928,57 @@
           <t>29/06/2026</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr"/>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>HUARI</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>HUARI</t>
+          <t>HUANTAR</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>HUANTAR</t>
+          <t>CHUCOS</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>CHUCOS</t>
+          <t>021008</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>021008</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL HUARI</t>
         </is>
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>UGEL HUARI</t>
+          <t>86432</t>
         </is>
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>86432</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y58" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z58" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -7103,20 +7041,24 @@
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>MORROPON</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>MORROPON</t>
+          <t>BUENOS AIRES</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -7126,35 +7068,30 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>BUENOS AIRES</t>
+          <t>200402</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
         <is>
-          <t>200402</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL MORROPÓN</t>
         </is>
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>UGEL MORROPÓN</t>
+          <t>408</t>
         </is>
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z59" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -7217,58 +7154,57 @@
           <t>29/06/2026</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr"/>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>SANTA</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>SANTA</t>
+          <t>NUEVO CHIMBOTE</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>NUEVO CHIMBOTE</t>
+          <t>TANGAY BAJO MOCHICA</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>TANGAY BAJO MOCHICA</t>
+          <t>021809</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
         <is>
-          <t>021809</t>
+          <t>DRE ANCASH</t>
         </is>
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>DRE ANCASH</t>
+          <t>UGEL SANTA</t>
         </is>
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>UGEL SANTA</t>
+          <t>88398</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>88398</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="Z60" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>
@@ -7331,10 +7267,14 @@
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PIURA</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
@@ -7344,45 +7284,40 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>PIURA</t>
+          <t>CATACAOS</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>CATACAOS</t>
+          <t>MONTE CASTILLO</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>MONTE CASTILLO</t>
+          <t>200105</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>200105</t>
+          <t>DRE PIURA</t>
         </is>
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>DRE PIURA</t>
+          <t>UGEL PIURA</t>
         </is>
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>UGEL PIURA</t>
+          <t>JOSE CARLOS MARIATEGUI LACHIRA</t>
         </is>
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>JOSE CARLOS MARIATEGUI LACHIRA</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="Y61" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="Z61" t="inlineStr">
         <is>
           <t>UGRD</t>
         </is>

</xml_diff>